<commit_message>
Separated clustering analyses into their own folder within the Zinc folder
</commit_message>
<xml_diff>
--- a/Copper/5. Statistical data analysis/Plots of Cu Toxicity/overlap_Cu_by_typology.xlsx
+++ b/Copper/5. Statistical data analysis/Plots of Cu Toxicity/overlap_Cu_by_typology.xlsx
@@ -1,52 +1,62 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ornl-my.sharepoint.com/personal/q4q_ornl_gov/Documents/Research/Bioavailability Project/BLM_spatial_assessmt/Copper/5. Statistical data analysis/Plots of Cu Toxicity/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="12" documentId="11_C2CE81AC8D187207F9E19C5F0634935499BFBBC0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A984086-CE3D-4F88-923A-11B98C76FDE2}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Overlap_Cu_by_Typology" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Overlap_Cu_by_Typology" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
-    <t xml:space="preserve">Typology</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Overlap_Chronic_Toxicity_Daphnia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Overlap_Acute_Toxicity_Daphnia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Overlap_Chronic_Toxicity_Minnow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Overlap_Acute_Toxicity_Minnow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NP Tribs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P Tribs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD Tribs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Main Stem</t>
+    <t>Typology</t>
+  </si>
+  <si>
+    <t>Overlap_Chronic_Toxicity_Daphnia</t>
+  </si>
+  <si>
+    <t>Overlap_Acute_Toxicity_Daphnia</t>
+  </si>
+  <si>
+    <t>Overlap_Chronic_Toxicity_Minnow</t>
+  </si>
+  <si>
+    <t>Overlap_Acute_Toxicity_Minnow</t>
+  </si>
+  <si>
+    <t>NP Tribs</t>
+  </si>
+  <si>
+    <t>P Tribs</t>
+  </si>
+  <si>
+    <t>PD Tribs</t>
+  </si>
+  <si>
+    <t>Main Stem</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="170" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -75,13 +85,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -363,11 +383,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="30.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.6328125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -384,74 +410,74 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="n">
-        <v>0.267485866425106</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.126085701419073</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="B2" s="1">
+        <v>0.26748586642510602</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.12608570141907299</v>
+      </c>
+      <c r="D2" s="1">
         <v>0.10937767298048</v>
       </c>
-      <c r="E2" t="n">
-        <v>0.0509304372161325</v>
+      <c r="E2" s="1">
+        <v>5.0930437216132503E-2</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="n">
-        <v>0.178112599232136</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.0653578127453638</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.0552145561993928</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.0233407296660637</v>
+      <c r="B3" s="1">
+        <v>0.17811259923213599</v>
+      </c>
+      <c r="C3" s="1">
+        <v>6.53578127453638E-2</v>
+      </c>
+      <c r="D3" s="1">
+        <v>5.5214556199392799E-2</v>
+      </c>
+      <c r="E3" s="1">
+        <v>2.3340729666063698E-2</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="1">
         <v>0.124657650785042</v>
       </c>
-      <c r="C4" t="n">
-        <v>0.0132961263838069</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.00616573745144461</v>
-      </c>
-      <c r="E4"/>
+      <c r="C4" s="1">
+        <v>1.32961263838069E-2</v>
+      </c>
+      <c r="D4" s="1">
+        <v>6.1657374514446101E-3</v>
+      </c>
+      <c r="E4" s="1"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="n">
-        <v>0.179232349726223</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.0335965484173412</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.021747051095094</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.00012070026478502</v>
+      <c r="B5" s="1">
+        <v>0.17923234972622301</v>
+      </c>
+      <c r="C5" s="1">
+        <v>3.35965484173412E-2</v>
+      </c>
+      <c r="D5" s="1">
+        <v>2.1747051095093999E-2</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1.2070026478501999E-4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>